<commit_message>
feat: update student write request and import service to allow optional fields for English names, phone, and email
</commit_message>
<xml_diff>
--- a/resources/templates/Import Student Template.xlsx
+++ b/resources/templates/Import Student Template.xlsx
@@ -137,82 +137,22 @@
     <t>ช่องทางการรับเข้า</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>ชื่อภาษาอังกฤษ</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-      </rPr>
-      <t>*</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>นามสกุลภาษาอังกฤษ</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-      </rPr>
-      <t>*</t>
-    </r>
+    <t>ชื่อภาษาอังกฤษ</t>
+  </si>
+  <si>
+    <t>นามสกุลภาษาอังกฤษ</t>
   </si>
   <si>
     <t>ความสัมพันธ์</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>เบอร์โทร</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-      </rPr>
-      <t>*</t>
-    </r>
+    <t>เบอร์โทร</t>
   </si>
   <si>
     <t>สถานะ</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>อีเมล</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-      </rPr>
-      <t>*</t>
-    </r>
+    <t>อีเมล</t>
   </si>
   <si>
     <r>

</xml_diff>

<commit_message>
feat: implement study semester handling and update related requests and services
</commit_message>
<xml_diff>
--- a/resources/templates/Import Student Template.xlsx
+++ b/resources/templates/Import Student Template.xlsx
@@ -12,35 +12,173 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="82">
   <si>
     <t>รหัสนิสิต</t>
   </si>
   <si>
+    <t>คำนำหน้า</t>
+  </si>
+  <si>
+    <t>แผนการเรียน</t>
+  </si>
+  <si>
     <t>ข้อมูลส่วนตัว</t>
   </si>
   <si>
-    <t>ปีเข้าเรียน (พ.ศ.)</t>
-  </si>
-  <si>
     <t>อาจารย์ที่ปรึกษา</t>
   </si>
   <si>
+    <t>ช่องทางการรับเข้า</t>
+  </si>
+  <si>
+    <t>โรงเรียน ม.ปลาย</t>
+  </si>
+  <si>
+    <t>ความสัมพันธ์</t>
+  </si>
+  <si>
+    <t>สถานะ</t>
+  </si>
+  <si>
+    <t>ปี</t>
+  </si>
+  <si>
+    <t>เทอม</t>
+  </si>
+  <si>
+    <t>ดร.</t>
+  </si>
+  <si>
+    <t>แผนสหกิจศึกษา</t>
+  </si>
+  <si>
+    <t>อ.ร้อยโทอนุมัติ อิงคนินันท์</t>
+  </si>
+  <si>
+    <t>Admission</t>
+  </si>
+  <si>
+    <t>โรงเรียนวัดศาลาตึก</t>
+  </si>
+  <si>
+    <t>ญาติ</t>
+  </si>
+  <si>
+    <t>กำลังศึกษา</t>
+  </si>
+  <si>
+    <t>ภาคต้น</t>
+  </si>
+  <si>
+    <t>นาง</t>
+  </si>
+  <si>
+    <t>แผนไม่สหกิจศึกษา</t>
+  </si>
+  <si>
+    <t>รศ.ดร.อมรฤทธิ์ พุทธิพิพัฒน์ขจร</t>
+  </si>
+  <si>
+    <t>Portfolio</t>
+  </si>
+  <si>
+    <t>โรงเรียนเฉลิมพระเกียรติสมเด็จพระศรีนครินทร์ กาญจนบุรี</t>
+  </si>
+  <si>
+    <t>บิดา</t>
+  </si>
+  <si>
+    <t>จบการศึกษา</t>
+  </si>
+  <si>
+    <t>ภาคปลาย</t>
+  </si>
+  <si>
+    <t>น.ส.</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.บุญรัตน์ เผดิมรอด</t>
+  </si>
+  <si>
+    <t>รับตรงร่วมกัน</t>
+  </si>
+  <si>
+    <t>พี่ชาย</t>
+  </si>
+  <si>
+    <t>พ้นสภาพนิสิต</t>
+  </si>
+  <si>
+    <t>การเข้าเรียน</t>
+  </si>
+  <si>
+    <t>ภาคฤดูร้อน</t>
+  </si>
+  <si>
+    <t>นาย</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.จักกริช พฤษการ</t>
+  </si>
+  <si>
+    <t>โควตา</t>
+  </si>
+  <si>
+    <t>พี่สาว</t>
+  </si>
+  <si>
+    <t>ผศ.</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.ดวงเพ็ญ เจตน์พิพัฒนพงษ์</t>
+  </si>
+  <si>
+    <t>มารดา</t>
+  </si>
+  <si>
     <t>ช่องทางรับเข้า</t>
   </si>
   <si>
-    <t>โรงเรียน ม.ปลาย</t>
-  </si>
-  <si>
     <t>ผู้ปกครอง</t>
   </si>
   <si>
-    <t>คำนำหน้า</t>
+    <t>รศ.</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.กายรัฐ เจริญราษฎร์</t>
+  </si>
+  <si>
+    <t>ศ.</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.พิเชษฐ์ สืบสายพรหม</t>
+  </si>
+  <si>
+    <t>อ.พฤษพล ตั้งสัจจะธรรม</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.ศิวดล เสถียรพัฒนากูล</t>
   </si>
   <si>
     <t>สถานะปัจจุบัน</t>
   </si>
   <si>
+    <t>ผศ.ดร.เสกสรรค์ มธุลาภรังสรรค์</t>
+  </si>
+  <si>
+    <t>รศ.ดร.ฐิติพงษ์ สถิรเมธีกุล</t>
+  </si>
+  <si>
+    <t>อ.ธีรวัฒน์ หวายฤทธิ์</t>
+  </si>
+  <si>
+    <t>ผศ.ดร.วรัญญา อรรถเสนา</t>
+  </si>
+  <si>
+    <t>อาจารย์จิรภัทร แซ่ลี้</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
@@ -59,13 +197,16 @@
     </r>
   </si>
   <si>
+    <t>เลขบัตรประชาชน</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>เลขบัตรประชาชน</t>
+      <t>คำนำหน้า</t>
     </r>
     <r>
       <rPr>
@@ -83,7 +224,7 @@
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>คำนำหน้า</t>
+      <t>ชื่อภาษาไทย</t>
     </r>
     <r>
       <rPr>
@@ -95,16 +236,13 @@
     </r>
   </si>
   <si>
-    <t>แผนการเรียน</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>ชื่อภาษาไทย</t>
+      <t>นามสกุลภาษาไทย</t>
     </r>
     <r>
       <rPr>
@@ -116,13 +254,25 @@
     </r>
   </si>
   <si>
+    <t>ชื่อภาษาอังกฤษ</t>
+  </si>
+  <si>
+    <t>นามสกุลภาษาอังกฤษ</t>
+  </si>
+  <si>
+    <t>เบอร์โทร</t>
+  </si>
+  <si>
+    <t>อีเมล</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>นามสกุลภาษาไทย</t>
+      <t>ปีเข้าเรียน (พ.ศ.)</t>
     </r>
     <r>
       <rPr>
@@ -134,34 +284,13 @@
     </r>
   </si>
   <si>
-    <t>ช่องทางการรับเข้า</t>
-  </si>
-  <si>
-    <t>ชื่อภาษาอังกฤษ</t>
-  </si>
-  <si>
-    <t>นามสกุลภาษาอังกฤษ</t>
-  </si>
-  <si>
-    <t>ความสัมพันธ์</t>
-  </si>
-  <si>
-    <t>เบอร์โทร</t>
-  </si>
-  <si>
-    <t>สถานะ</t>
-  </si>
-  <si>
-    <t>อีเมล</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>ปีเข้าเรียน (พ.ศ.)</t>
+      <t>ปี</t>
     </r>
     <r>
       <rPr>
@@ -173,15 +302,30 @@
     </r>
   </si>
   <si>
-    <t>ดร.</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
         <b/>
         <color theme="1"/>
       </rPr>
+      <t>เทอม</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color rgb="FFFF0000"/>
+      </rPr>
+      <t>*</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
       <t>ช่องทางรับเข้า</t>
     </r>
     <r>
@@ -194,36 +338,18 @@
     </r>
   </si>
   <si>
-    <t>แผนสหกิจศึกษา</t>
-  </si>
-  <si>
     <t>คำนำหน้าผู้ปกครอง</t>
   </si>
   <si>
-    <t>อ.ร้อยโทอนุมัติ อิงคนินันท์</t>
-  </si>
-  <si>
     <t>ชื่อผู้ปกครอง</t>
   </si>
   <si>
-    <t>Admission</t>
-  </si>
-  <si>
     <t>นามสกุลผู้ปกครอง</t>
   </si>
   <si>
-    <t>โรงเรียนวัดศาลาตึก</t>
-  </si>
-  <si>
-    <t>ญาติ</t>
-  </si>
-  <si>
     <t>เบอร์โทรผู้ปกครอง</t>
   </si>
   <si>
-    <t>กำลังศึกษา</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
@@ -242,60 +368,12 @@
     </r>
   </si>
   <si>
-    <t>นาง</t>
-  </si>
-  <si>
-    <t>แผนไม่สหกิจศึกษา</t>
-  </si>
-  <si>
-    <t>รศ.ดร.อมรฤทธิ์ พุทธิพิพัฒน์ขจร</t>
-  </si>
-  <si>
-    <t>Portfolio</t>
-  </si>
-  <si>
-    <t>โรงเรียนเฉลิมพระเกียรติสมเด็จพระศรีนครินทร์ กาญจนบุรี</t>
-  </si>
-  <si>
-    <t>บิดา</t>
-  </si>
-  <si>
-    <t>จบการศึกษา</t>
-  </si>
-  <si>
-    <t>น.ส.</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.บุญรัตน์ เผดิมรอด</t>
-  </si>
-  <si>
-    <t>รับตรงร่วมกัน</t>
-  </si>
-  <si>
-    <t>พี่ชาย</t>
-  </si>
-  <si>
-    <t>พ้นสภาพนิสิต</t>
-  </si>
-  <si>
-    <t>นาย</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.จักกริช พฤษการ</t>
-  </si>
-  <si>
     <t>นิสิต</t>
   </si>
   <si>
-    <t>โควตา</t>
-  </si>
-  <si>
     <t>ทดสอบ</t>
   </si>
   <si>
-    <t>พี่สาว</t>
-  </si>
-  <si>
     <t>Student</t>
   </si>
   <si>
@@ -305,58 +383,16 @@
     <t>0981112233</t>
   </si>
   <si>
-    <t>ผศ.</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.ดวงเพ็ญ เจตน์พิพัฒนพงษ์</t>
-  </si>
-  <si>
-    <t>มารดา</t>
-  </si>
-  <si>
     <t>test@gmail.com</t>
   </si>
   <si>
-    <t>รศ.</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.กายรัฐ เจริญราษฎร์</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.วรัญญา อรรถเสนา</t>
-  </si>
-  <si>
-    <t>ศ.</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.พิเชษฐ์ สืบสายพรหม</t>
-  </si>
-  <si>
-    <t>อ.พฤษพล ตั้งสัจจะธรรม</t>
-  </si>
-  <si>
-    <t>ผศ.ดร.ศิวดล เสถียรพัฒนากูล</t>
-  </si>
-  <si>
     <t>ใจดี</t>
   </si>
   <si>
     <t>จริงใจ</t>
   </si>
   <si>
-    <t>ผศ.ดร.เสกสรรค์ มธุลาภรังสรรค์</t>
-  </si>
-  <si>
-    <t>รศ.ดร.ฐิติพงษ์ สถิรเมธีกุล</t>
-  </si>
-  <si>
     <t>0842331123</t>
-  </si>
-  <si>
-    <t>อ.ธีรวัฒน์ หวายฤทธิ์</t>
-  </si>
-  <si>
-    <t>อาจารย์จิรภัทร แซ่ลี้</t>
   </si>
 </sst>
 </file>
@@ -376,12 +412,12 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
-    <font/>
     <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font/>
   </fonts>
   <fills count="4">
     <fill>
@@ -457,21 +493,21 @@
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -704,193 +740,214 @@
     <col customWidth="1" min="8" max="8" width="16.5"/>
     <col customWidth="1" min="9" max="9" width="26.88"/>
     <col customWidth="1" min="10" max="10" width="18.38"/>
-    <col customWidth="1" min="11" max="11" width="25.13"/>
-    <col customWidth="1" min="12" max="12" width="21.88"/>
-    <col customWidth="1" min="13" max="13" width="30.13"/>
-    <col customWidth="1" min="14" max="14" width="16.13"/>
-    <col customWidth="1" min="16" max="16" width="16.88"/>
-    <col customWidth="1" min="17" max="17" width="16.25"/>
-    <col customWidth="1" min="18" max="18" width="16.13"/>
-    <col customWidth="1" min="19" max="19" width="19.5"/>
+    <col customWidth="1" min="11" max="13" width="25.13"/>
+    <col customWidth="1" min="14" max="14" width="21.88"/>
+    <col customWidth="1" min="15" max="15" width="30.13"/>
+    <col customWidth="1" min="16" max="16" width="16.13"/>
+    <col customWidth="1" min="18" max="18" width="16.88"/>
+    <col customWidth="1" min="19" max="19" width="16.25"/>
+    <col customWidth="1" min="20" max="20" width="16.13"/>
+    <col customWidth="1" min="21" max="21" width="19.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="5"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="N1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="1" t="s">
-        <v>8</v>
+      <c r="P1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q1" s="5"/>
+      <c r="R1" s="5"/>
+      <c r="S1" s="5"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="A2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>6.020501112E9</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1.709800313999E12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J3" s="3">
+        <v>2569.0</v>
+      </c>
+      <c r="K3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="O3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="U3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6">
-        <v>6.020501112E9</v>
-      </c>
-      <c r="B3" s="6">
-        <v>1.709800313999E12</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="J3" s="6">
-        <v>2569.0</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>34</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="B1:I1"/>
-    <mergeCell ref="N1:R1"/>
+    <mergeCell ref="P1:T1"/>
+    <mergeCell ref="J1:L1"/>
   </mergeCells>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K3">
+      <formula1>MasterData!$H$2:$H$9</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M3">
       <formula1>MasterData!$C$2:$C$1048576</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="O3">
       <formula1>MasterData!$E$2:$E$1048576</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="S3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="U3">
       <formula1>MasterData!$G$2:$G$1048576</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3 N3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3 P3">
       <formula1>MasterData!$A$2:$A$1048576</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L3">
+      <formula1>MasterData!$I$2:$I$4</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N3">
       <formula1>MasterData!$D$2:$D$1048576</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Q3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="S3">
       <formula1>MasterData!$F$2:$F$1048576</formula1>
     </dataValidation>
   </dataValidations>
@@ -913,165 +970,204 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="G1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="5" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="C3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="F3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="H3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="C4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" s="6" t="s">
+      <c r="H4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="C5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="F5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="H5" s="3">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
+      <c r="H6" s="3">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="H7" s="3">
+        <v>6.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="C8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H8" s="3">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
+      <c r="H9" s="3">
+        <v>8.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="C10" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" s="6" t="s">
+    </row>
+    <row r="11">
+      <c r="C11" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="6" t="s">
+    </row>
+    <row r="13">
+      <c r="C13" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="3" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="C9" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="C11" s="6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="C12" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="C13" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
     <row r="15">
-      <c r="C15" s="6" t="s">
-        <v>74</v>
+      <c r="C15" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>